<commit_message>
process list bug fixed
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_helper.xlsx
+++ b/output_data/vt_DE_helper.xlsx
@@ -8495,6 +8495,11 @@
           <t>helper_pow_exo_sec_elec</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H15" t="inlineStr">
         <is>
           <t>exo_sec_elec</t>
@@ -8517,6 +8522,11 @@
           <t>helper_pow_ind_biomass</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H16" t="inlineStr">
         <is>
           <t>iip_chemi_biomass</t>
@@ -8566,6 +8576,11 @@
           <t>helper_source_env</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H18" t="inlineStr">
         <is>
           <t>pri_envir_heat</t>
@@ -8588,6 +8603,11 @@
           <t>helper_source_geo</t>
         </is>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H19" t="inlineStr">
         <is>
           <t>pri_geoth_heat</t>
@@ -8610,6 +8630,11 @@
           <t>helper_source_marine</t>
         </is>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H20" t="inlineStr">
         <is>
           <t>pri_marine</t>
@@ -8632,6 +8657,11 @@
           <t>helper_source_saving</t>
         </is>
       </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H21" t="inlineStr">
         <is>
           <t>sec_saving</t>
@@ -8654,6 +8684,11 @@
           <t>helper_source_solar_radiation</t>
         </is>
       </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H22" t="inlineStr">
         <is>
           <t>pri_solar_radiation</t>
@@ -8676,6 +8711,11 @@
           <t>helper_source_wind</t>
         </is>
       </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H23" t="inlineStr">
         <is>
           <t>pri_wind_energy</t>
@@ -8698,6 +8738,11 @@
           <t>helper_x2x_heating_oil</t>
         </is>
       </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H24" t="inlineStr">
         <is>
           <t>sec_heating_oil</t>
@@ -9071,6 +9116,11 @@
           <t>helper_x2x_storage_crude_oil</t>
         </is>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H38" t="inlineStr">
         <is>
           <t>pri_crude_oil</t>
@@ -9093,6 +9143,11 @@
           <t>helper_x2x_storage_diesel</t>
         </is>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr">
         <is>
           <t>sec_diesel</t>
@@ -9115,6 +9170,11 @@
           <t>helper_x2x_storage_gasoline</t>
         </is>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>notFound</t>
+        </is>
+      </c>
       <c r="H40" t="inlineStr">
         <is>
           <t>sec_gasoline</t>
@@ -9162,6 +9222,11 @@
       <c r="C42" t="inlineStr">
         <is>
           <t>helper_x2x_storage_kerosene</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>notFound</t>
         </is>
       </c>
       <c r="H42" t="inlineStr">

</xml_diff>

<commit_message>
update MATI in primary_cg
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_helper.xlsx
+++ b/output_data/vt_DE_helper.xlsx
@@ -15016,7 +15016,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>NRGI</t>
+          <t>MATI</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
@@ -15043,7 +15043,7 @@
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>NRGI</t>
+          <t>MATI</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
@@ -15070,7 +15070,7 @@
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>NRGI</t>
+          <t>MATI</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">

</xml_diff>

<commit_message>
update commodity_list and process_list
</commit_message>
<xml_diff>
--- a/output_data/vt_DE_helper.xlsx
+++ b/output_data/vt_DE_helper.xlsx
@@ -5141,34 +5141,34 @@
       <c r="H93" s="7" t="inlineStr"/>
       <c r="I93" s="7" t="inlineStr"/>
       <c r="J93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="K93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="L93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="M93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="N93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="O93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="P93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="Q93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="R93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
       <c r="S93" s="7" t="n">
-        <v>0.0036</v>
+        <v>1</v>
       </c>
     </row>
     <row r="94">
@@ -11722,17 +11722,17 @@
     <row r="4">
       <c r="B4" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>sec_naphtha_orig</t>
+          <t>emi_co2_neg_fuel_cc_pow</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -11744,34 +11744,34 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>pri_marine_f</t>
+          <t>iip_heat_proc</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="B6" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>exo_sec_elec_b</t>
+          <t>sec_lpg</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -11783,17 +11783,12 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>iip_heat_proc</t>
+          <t>pri_solar_radiation_a</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -11805,12 +11800,12 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>sec_naphtha</t>
+          <t>sec_ammonia_orig</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -11822,24 +11817,19 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>pri_wind_energy_f</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>PJ/PJ</t>
+          <t>pri_crude_oil</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="B10" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>iip_chemi_lpg</t>
+          <t>pri_wind_energy_e</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -11856,12 +11846,17 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>sec_kerosene_syn_orig</t>
+          <t>pri_geoth_heat</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -11873,17 +11868,12 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_g</t>
+          <t>sec_diesel_fos_orig</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -11895,12 +11885,12 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_c</t>
+          <t>pri_geoth_heat_b</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
@@ -11917,56 +11907,51 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_f</t>
+          <t>pri_wind_energy</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="B15" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>iip_chemi_methanol</t>
+          <t>exo_sec_elec_e</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>Mt/Mt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="B16" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>exo_sec_elec_e</t>
+          <t>iip_chemi_methanol</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>Mt</t>
         </is>
       </c>
     </row>
@@ -11978,12 +11963,12 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_f</t>
+          <t>sec_kerosene_orig</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -11995,17 +11980,17 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>pri_geoth_heat</t>
+          <t>sec_elec_b</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>HTHEAT</t>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12017,12 +12002,12 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>pri_marine</t>
+          <t>sec_hydrogen</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12034,12 +12019,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_g</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>PJ/PJ</t>
+          <t>sec_gasoline</t>
         </is>
       </c>
     </row>
@@ -12051,17 +12031,12 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>sec_elec_ind</t>
+          <t>iip_steel_blafu_gas_in</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
           <t>PJ</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12073,12 +12048,12 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>sec_diesel_orig</t>
+          <t>sec_naphtha_syn_orig</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12090,12 +12065,12 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>sec_lpg</t>
+          <t>sec_diesel_syn_orig</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12107,12 +12082,17 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>sec_methanol_orig</t>
+          <t>sec_elec_e</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12124,29 +12104,34 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>sec_biomethanol_orig</t>
+          <t>iip_auto_space_heat</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>sec_naphtha_fos_orig</t>
+          <t>iip_chemi_nh3</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>Mt</t>
         </is>
       </c>
     </row>
@@ -12158,12 +12143,12 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>sec_syngas</t>
+          <t>pri_natural_gas</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12175,51 +12160,46 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>sec_hydrogen</t>
-        </is>
-      </c>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>PJ/PJ</t>
+          <t>sec_saving</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="B29" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_b</t>
+          <t>exo_sec_elec_c</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="B30" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_d</t>
+          <t>emi_co2_neg_proc_cc_ind</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I30" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -12231,12 +12211,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>pri_marine_d</t>
+          <t>sec_gasoline_fos_orig</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12248,12 +12228,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_c</t>
+          <t>sec_naphtha_orig</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12265,12 +12245,12 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>emi_co2_neg_fuel_cc_x2x</t>
+          <t>emi_co2_neg_fuel_cc_ind</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PJ, Mt</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -12282,56 +12262,56 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>sec_elec</t>
+          <t>pri_geoth_heat_c</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>ELC</t>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="B35" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>exo_sec_elec_a</t>
+          <t>pri_geoth_heat_e</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>ELC</t>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="B36" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>ENV</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>sec_natural_gas_syn</t>
+          <t>emi_co2_neg_fuel_cc_x2x</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -12343,29 +12323,34 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>sec_gasoline_orig</t>
+          <t>pri_wind_energy_a</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="B38" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>iip_chemi_heavy_fuel_oil</t>
+          <t>exo_sec_elec_d</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12377,41 +12362,46 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>sec_kerosene_orig</t>
+          <t>pri_marine_g</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="B40" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>iip_chemi_steam</t>
+          <t>exo_sec_elec_b</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="B41" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>iip_chemi_methane</t>
+          <t>sec_methane_orig</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -12428,46 +12418,51 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>sec_gasoline_syn_orig</t>
+          <t>sec_biodiesel_orig</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="B43" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>iip_steel_blafu_gas</t>
+          <t>emi_co2_neg_air_dacc</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="B44" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>iip_chemi_biomethanol</t>
+          <t>sec_elec_d</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Mt/Mt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12479,56 +12474,46 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sec_elec_e</t>
+          <t>iip_chemi_steam</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I45" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="B46" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sec_elec_distr</t>
+          <t>iip_chemi_biomethanol</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I46" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>Mt</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="B47" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>emi_co2_neg_air_dacc</t>
+          <t>sec_naphtha_fos_orig</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>PJ, Mt</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12540,34 +12525,34 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>sec_elec_f</t>
+          <t>pri_geoth_heat_g</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>ELC</t>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="B49" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_a</t>
+          <t>iip_chemi_mtg_mtk_h2</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12579,7 +12564,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>iip_steel_coke_oven_gas_in</t>
+          <t>sec_kerosene_syn_orig</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
@@ -12596,12 +12581,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>exo_sec_elec_d</t>
+          <t>exo_sec_elec</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
@@ -12618,7 +12603,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>sec_kerosene</t>
+          <t>sec_kerosene_fos_orig</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12630,73 +12620,68 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>pri_marine_c</t>
+          <t>sec_syngas_sr</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="B54" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>iip_elec</t>
+          <t>emi_co2_stored</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I54" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="B55" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>exo_sec_elec_f</t>
+          <t>iip_chemi_nh3_h2</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I55" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="B56" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>iip_chemi_biomass</t>
+          <t>sec_elec_g</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -12708,12 +12693,17 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>sec_gasoline_fos_orig</t>
+          <t>pri_geoth_heat_a</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -12725,29 +12715,29 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>pri_marine_a</t>
+          <t>pri_wind_energy_d</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="B59" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_e</t>
+          <t>iip_chemi_meoh_h2</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12759,29 +12749,29 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>sec_ammonia_orig</t>
+          <t>pri_marine_c</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>PJ/Mt</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="B61" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>exo_sec_elec</t>
+          <t>sec_elec_c</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -12793,12 +12783,12 @@
     <row r="62">
       <c r="B62" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>iip_auto_space_heat</t>
+          <t>exo_sec_elec_a</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -12808,24 +12798,24 @@
       </c>
       <c r="I62" t="inlineStr">
         <is>
-          <t>HTHEAT</t>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="B63" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>pri_solar_radiation_d</t>
+          <t>iip_chemi_heavy_fuel_oil</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12837,12 +12827,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>pri_marine_b</t>
+          <t>pri_wind_energy_c</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12854,7 +12844,17 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>pri_crude_oil</t>
+          <t>pri_geoth_heat_f</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -12866,46 +12866,41 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>sec_methane_orig</t>
+          <t>pri_solar_radiation_g</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="B67" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>emi_co2_reusable</t>
-        </is>
-      </c>
-      <c r="E67" t="inlineStr">
-        <is>
-          <t>Kt/Kt</t>
+          <t>sec_heating_oil</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="B68" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>sec_kerosene_fos_orig</t>
+          <t>iip_chemi_lpg</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12917,29 +12912,29 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>pri_solar_radiation</t>
+          <t>pri_wind_energy_g</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="B70" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>sec_naphtha_syn_orig</t>
+          <t>iip_chemi_biomass</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12951,17 +12946,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>sec_elec_a</t>
+          <t>iip_steel_coke_oven_gas_in</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I71" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12973,7 +12963,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>sec_gasoline</t>
+          <t>sec_biomethanol_orig</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -12985,12 +12980,7 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>iip_steel_blafu_gas_in</t>
-        </is>
-      </c>
-      <c r="E73" t="inlineStr">
-        <is>
-          <t>PJ</t>
+          <t>sec_kerosene</t>
         </is>
       </c>
     </row>
@@ -13002,17 +12992,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_a</t>
+          <t>sec_heavy_fuel_oil</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13024,17 +13009,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>sec_elec_b</t>
+          <t>pri_solar_radiation_f</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I75" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13046,12 +13026,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>sec_heavy_fuel_oil</t>
+          <t>sec_diesel_orig</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13063,12 +13043,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>sec_syngas_sr</t>
+          <t>pri_marine_a</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13080,34 +13060,29 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>sec_methane</t>
+          <t>pri_solar_radiation_b</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="B79" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_e</t>
+          <t>iip_chemi_methane</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I79" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13119,12 +13094,12 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>pri_wind_energy_c</t>
+          <t>pri_solar_radiation_d</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13136,17 +13111,12 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>pri_geoth_heat_b</t>
+          <t>sec_gasoline_orig</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I81" t="inlineStr">
-        <is>
-          <t>HTHEAT</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13158,12 +13128,12 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>sec_diesel_syn_orig</t>
+          <t>pri_solar_radiation</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13175,24 +13145,24 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>pri_marine_e</t>
+          <t>pri_wind_energy_f</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="B84" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>iip_chemi_mtg_mtk_h2</t>
+          <t>pri_marine_e</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -13204,34 +13174,44 @@
     <row r="85">
       <c r="B85" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>iip_chemi_meoh_h2</t>
+          <t>sec_elec_f</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
           <t>PJ</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="B86" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>emi_co2_neg_fuel_cc_pow</t>
+          <t>exo_sec_elec_g</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>PJ, Mt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13243,12 +13223,12 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>iip_steel_coke_oven_gas</t>
+          <t>sec_gasoline_syn_orig</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13260,29 +13240,29 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>pri_wind_energy_b</t>
-        </is>
-      </c>
-      <c r="E88" t="inlineStr">
-        <is>
-          <t>PJ/PJ</t>
+          <t>sec_diesel</t>
         </is>
       </c>
     </row>
     <row r="89">
       <c r="B89" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>emi_co2_neg_proc_cc_ind</t>
+          <t>pri_geoth_heat_d</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>kt/Kt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -13294,7 +13274,12 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>sec_heating_oil</t>
+          <t>iip_steel_blafu_gas</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13306,24 +13291,39 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>sec_saving</t>
+          <t>sec_elec_distr</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="B92" t="inlineStr">
         <is>
-          <t>ENV</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>emi_co2_neg_fuel_cc_ind</t>
+          <t>sec_elec</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>kt/Kt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13340,41 +13340,36 @@
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="94">
       <c r="B94" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>exo_sec_elec_g</t>
+          <t>pri_wind_energy_b</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I94" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="95">
       <c r="B95" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>iip_chemi_naphtha</t>
+          <t>sec_methane</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
@@ -13391,29 +13386,29 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>pri_wind_energy_a</t>
+          <t>pri_marine_b</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="B97" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>pri_natural_gas</t>
+          <t>iip_chemi_naphtha</t>
         </is>
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13425,12 +13420,12 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>sec_diesel_fos_orig</t>
+          <t>iip_steel_coke_oven_gas</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13442,17 +13437,12 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>sec_elec_g</t>
+          <t>pri_solar_radiation_c</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I99" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13464,12 +13454,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>pri_marine_g</t>
+          <t>pri_marine</t>
         </is>
       </c>
       <c r="E100" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13481,39 +13471,29 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>sec_elec_d</t>
+          <t>sec_naphtha</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I101" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="B102" t="inlineStr">
         <is>
-          <t>DEM</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>exo_sec_elec_c</t>
+          <t>pri_solar_radiation_e</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I102" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13525,12 +13505,17 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>pri_wind_energy</t>
+          <t>iip_elec</t>
         </is>
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13542,29 +13527,34 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>sec_biodiesel_orig</t>
+          <t>sec_methanol_orig</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="B105" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>DEM</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>pri_wind_energy_g</t>
+          <t>exo_sec_elec_f</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13576,24 +13566,24 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>pri_wind_energy_d</t>
+          <t>sec_syngas</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="B107" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>iip_chemi_nh3_h2</t>
+          <t>pri_bio_wood</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -13605,17 +13595,17 @@
     <row r="108">
       <c r="B108" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>iip_chemi_nh3</t>
+          <t>pri_marine_f</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Mt/Mt</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13627,17 +13617,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>sec_elec_c</t>
+          <t>pri_marine_d</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
-        </is>
-      </c>
-      <c r="I109" t="inlineStr">
-        <is>
-          <t>ELC</t>
+          <t>PJ</t>
         </is>
       </c>
     </row>
@@ -13649,29 +13634,34 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>pri_envir_heat</t>
+          <t>sec_elec_a</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
         <is>
-          <t>HTHEAT</t>
+          <t>ELC</t>
         </is>
       </c>
     </row>
     <row r="111">
       <c r="B111" t="inlineStr">
         <is>
-          <t>MAT</t>
+          <t>NRG</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>emi_co2_stored</t>
-        </is>
-      </c>
-      <c r="E111" t="inlineStr">
-        <is>
-          <t>Kt</t>
+          <t>pri_envir_heat</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>HTHEAT</t>
         </is>
       </c>
     </row>
@@ -13683,12 +13673,17 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>pri_bio_wood</t>
+          <t>sec_elec_ind</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>ELC</t>
         </is>
       </c>
     </row>
@@ -13700,24 +13695,29 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>sec_diesel</t>
+          <t>sec_natural_gas_syn</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="B114" t="inlineStr">
         <is>
-          <t>NRG</t>
+          <t>MAT</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>pri_wind_energy_e</t>
+          <t>emi_co2_reusable</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>Kt</t>
         </is>
       </c>
     </row>
@@ -13813,12 +13813,12 @@
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>Capacity Unit</t>
+          <t>PJ</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -13850,7 +13850,12 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
@@ -13877,7 +13882,12 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -13904,7 +13914,12 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -13931,7 +13946,12 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
@@ -13958,7 +13978,12 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -13985,7 +14010,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
@@ -14012,7 +14042,12 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
@@ -14039,7 +14074,12 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -14066,7 +14106,12 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
@@ -14093,7 +14138,12 @@
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
@@ -14120,7 +14170,12 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
@@ -14147,7 +14202,12 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
@@ -14174,7 +14234,12 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
@@ -14201,7 +14266,12 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
@@ -14228,7 +14298,12 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
@@ -14255,7 +14330,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
@@ -14282,7 +14362,12 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
@@ -14309,7 +14394,12 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
@@ -14336,7 +14426,12 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
@@ -14363,7 +14458,12 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
@@ -14390,7 +14490,12 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H24" t="inlineStr">
@@ -14417,7 +14522,12 @@
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
@@ -14444,7 +14554,12 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -14471,7 +14586,12 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H27" t="inlineStr">
@@ -14498,7 +14618,12 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H28" t="inlineStr">
@@ -14525,7 +14650,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H29" t="inlineStr">
@@ -14552,7 +14682,12 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H30" t="inlineStr">
@@ -14579,7 +14714,12 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H31" t="inlineStr">
@@ -14606,7 +14746,12 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H32" t="inlineStr">
@@ -14633,7 +14778,12 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H33" t="inlineStr">
@@ -14660,7 +14810,12 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H34" t="inlineStr">
@@ -14687,7 +14842,12 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H35" t="inlineStr">
@@ -14714,7 +14874,12 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H36" t="inlineStr">
@@ -14741,7 +14906,12 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H37" t="inlineStr">
@@ -14768,7 +14938,12 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H38" t="inlineStr">
@@ -14795,7 +14970,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>Kt/Kt</t>
+          <t>kt</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>Kt</t>
         </is>
       </c>
       <c r="H39" t="inlineStr">
@@ -14822,6 +15002,11 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>kt</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
           <t>Kt</t>
         </is>
       </c>
@@ -14852,6 +15037,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H41" t="inlineStr">
         <is>
           <t>iip_auto_space_heat</t>
@@ -14879,6 +15069,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H42" t="inlineStr">
         <is>
           <t>iip_chemi_steam</t>
@@ -14906,6 +15101,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H43" t="inlineStr">
         <is>
           <t>sec_elec_ind</t>
@@ -14933,6 +15133,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H44" t="inlineStr">
         <is>
           <t>iip_steel_blafu_gas_in</t>
@@ -14960,6 +15165,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H45" t="inlineStr">
         <is>
           <t>iip_steel_coke_oven_gas_in</t>
@@ -14984,7 +15194,12 @@
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H46" t="inlineStr">
@@ -15011,7 +15226,12 @@
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H47" t="inlineStr">
@@ -15038,7 +15258,12 @@
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F48" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H48" t="inlineStr">
@@ -15065,7 +15290,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>PJ/Mt</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F49" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H49" t="inlineStr">
@@ -15092,7 +15322,12 @@
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H50" t="inlineStr">
@@ -15119,7 +15354,12 @@
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H51" t="inlineStr">
@@ -15146,7 +15386,12 @@
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H52" t="inlineStr">
@@ -15176,6 +15421,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr">
         <is>
           <t>sec_elec_ind</t>
@@ -15203,6 +15453,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H54" t="inlineStr">
         <is>
           <t>iip_chemi_biomass</t>
@@ -15227,7 +15482,12 @@
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H55" t="inlineStr">
@@ -15254,7 +15514,12 @@
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H56" t="inlineStr">
@@ -15281,7 +15546,12 @@
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H57" t="inlineStr">
@@ -15308,7 +15578,12 @@
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H58" t="inlineStr">
@@ -15335,7 +15610,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H59" t="inlineStr">
@@ -15362,7 +15642,12 @@
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H60" t="inlineStr">
@@ -15389,7 +15674,12 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H61" t="inlineStr">
@@ -15419,6 +15709,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr">
         <is>
           <t>iip_chemi_heavy_fuel_oil</t>
@@ -15446,6 +15741,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr">
         <is>
           <t>iip_chemi_lpg</t>
@@ -15473,6 +15773,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H64" t="inlineStr">
         <is>
           <t>iip_chemi_meoh_h2</t>
@@ -15500,6 +15805,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H65" t="inlineStr">
         <is>
           <t>iip_chemi_methane</t>
@@ -15527,6 +15837,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H66" t="inlineStr">
         <is>
           <t>iip_chemi_mtg_mtk_h2</t>
@@ -15554,6 +15869,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H67" t="inlineStr">
         <is>
           <t>iip_chemi_naphtha</t>
@@ -15581,6 +15901,11 @@
           <t>PJ</t>
         </is>
       </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>PJ</t>
+        </is>
+      </c>
       <c r="H68" t="inlineStr">
         <is>
           <t>iip_chemi_nh3_h2</t>
@@ -15605,7 +15930,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H69" t="inlineStr">
@@ -15632,7 +15962,12 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H70" t="inlineStr">
@@ -15659,7 +15994,12 @@
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H71" t="inlineStr">
@@ -15686,7 +16026,12 @@
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H72" t="inlineStr">
@@ -15713,7 +16058,12 @@
       </c>
       <c r="E73" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H73" t="inlineStr">
@@ -15740,7 +16090,12 @@
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H74" t="inlineStr">
@@ -15767,7 +16122,12 @@
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H75" t="inlineStr">
@@ -15794,7 +16154,12 @@
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H76" t="inlineStr">
@@ -15821,7 +16186,12 @@
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H77" t="inlineStr">
@@ -15848,7 +16218,12 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>PJ/PJ</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H78" t="inlineStr">
@@ -15875,7 +16250,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>notFound</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>GWh</t>
         </is>
       </c>
       <c r="H79" t="inlineStr">
@@ -15902,7 +16282,12 @@
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>MWh</t>
+          <t>PJ</t>
+        </is>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>PJ</t>
         </is>
       </c>
       <c r="H80" t="inlineStr">

</xml_diff>